<commit_message>
se empezo a dividr el procesamiento de esp32- android y pc
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_esp32_android.xlsx
+++ b/medidor de metricas/automatizacion_completa/datos_entrada/datos_entrada_esp32_android.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\medidor de metricas\automatizacion_completa\datos_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE06E3C-9758-4E0E-92B6-F37A5854BE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5F7DFF-4C69-4D7E-8F2A-681000ECCBBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="32">
   <si>
     <t>Codigo</t>
   </si>
@@ -128,37 +128,7 @@
     <t>L2-1C2026-AND-V</t>
   </si>
   <si>
-    <t>0.9%</t>
-  </si>
-  <si>
-    <t>1.3%</t>
-  </si>
-  <si>
-    <t>1.4%</t>
-  </si>
-  <si>
-    <t>1.5%</t>
-  </si>
-  <si>
-    <t>2.4%</t>
-  </si>
-  <si>
     <t>leyendo GPS</t>
-  </si>
-  <si>
-    <t>18.35%</t>
-  </si>
-  <si>
-    <t>27.6%</t>
-  </si>
-  <si>
-    <t>1.6%</t>
-  </si>
-  <si>
-    <t>1.05%</t>
-  </si>
-  <si>
-    <t>0.83%</t>
   </si>
   <si>
     <t>Context Windows</t>
@@ -168,8 +138,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -195,7 +166,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,12 +199,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -257,7 +222,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -294,20 +259,10 @@
     <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
@@ -599,11 +554,11 @@
       <c r="H2" s="12">
         <v>0.01</v>
       </c>
-      <c r="I2" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="19" t="s">
-        <v>32</v>
+      <c r="I2" s="14">
+        <v>103</v>
+      </c>
+      <c r="J2" s="14">
+        <v>111</v>
       </c>
       <c r="K2" s="11">
         <v>7792</v>
@@ -634,11 +589,11 @@
       <c r="H3" s="12">
         <v>0.01</v>
       </c>
-      <c r="I3" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" s="19" t="s">
-        <v>33</v>
+      <c r="I3" s="14">
+        <v>104</v>
+      </c>
+      <c r="J3" s="14">
+        <v>123</v>
       </c>
       <c r="K3" s="11">
         <v>7792</v>
@@ -660,22 +615,22 @@
       <c r="E4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="15">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" s="18">
+      <c r="H4" s="12">
+        <v>0.27</v>
+      </c>
+      <c r="I4" s="14">
+        <v>92</v>
+      </c>
+      <c r="J4" s="14">
+        <v>116</v>
+      </c>
+      <c r="K4" s="14">
         <v>1114</v>
       </c>
     </row>
@@ -695,22 +650,22 @@
       <c r="E5" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>34</v>
+      <c r="F5" s="15">
+        <v>2.4E-2</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="J5" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="18">
+        <v>30</v>
+      </c>
+      <c r="H5" s="12">
+        <v>0.18</v>
+      </c>
+      <c r="I5" s="14">
+        <v>181</v>
+      </c>
+      <c r="J5" s="14">
+        <v>185</v>
+      </c>
+      <c r="K5" s="14">
         <v>1114</v>
       </c>
     </row>
@@ -719,72 +674,72 @@
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
       <c r="E6" s="11"/>
-      <c r="F6" s="14"/>
+      <c r="F6" s="12"/>
       <c r="G6" s="13"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="18"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11">
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
       <c r="E7" s="11"/>
-      <c r="F7" s="14"/>
+      <c r="F7" s="12"/>
       <c r="G7" s="13"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
     </row>
     <row r="8" spans="1:11">
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11"/>
-      <c r="F8" s="15"/>
+      <c r="F8" s="12"/>
       <c r="G8" s="13"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="18"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
     </row>
     <row r="9" spans="1:11">
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11"/>
-      <c r="F9" s="15"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="13"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="18"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
     </row>
     <row r="10" spans="1:11">
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11"/>
-      <c r="F10" s="14"/>
+      <c r="F10" s="12"/>
       <c r="G10" s="13"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
     </row>
     <row r="11" spans="1:11">
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="16"/>
+      <c r="F11" s="12"/>
       <c r="G11" s="13"/>
-      <c r="H11" s="16"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="18"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -963,7 +918,7 @@
         <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C3" s="7">
         <v>2</v>

</xml_diff>